<commit_message>
Justify engineering explanations and long equipment text
Apply full-width alignment to document paragraphs and drawing captions, and to long XLSX text cells. Make the RF branch explanation wrap naturally and re-export the validated submission package.
</commit_message>
<xml_diff>
--- a/equipment/bill-of-materials.xlsx
+++ b/equipment/bill-of-materials.xlsx
@@ -130,7 +130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -158,6 +158,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -568,12 +574,12 @@
           <t>АФУ</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="10" t="inlineStr">
         <is>
           <t>In06_Потолочная, омни, MIMO, 800-2700 (G= 3dBi, H=360°)</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="10" t="inlineStr">
         <is>
           <t>Потолочная omni, MIMO; 800–2700 МГц; G=3 dBi; H=360°. Вертикальная диаграмма не предоставлена.</t>
         </is>
@@ -593,12 +599,12 @@
           <t>АФУ</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>PC211 Триплексер 1710-1880/1920-2170/2500-2690 МГц, одинарный, 4.3-10F, -160дБн, IP67</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>Триплексер 1710–1880 / 1920–2170 / 2500–2690 МГц, одинарный; 4.3-10F; IP67. Insertion loss не дано.</t>
         </is>
@@ -618,12 +624,12 @@
           <t>АФУ</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>PC221_Гибридный комбайнер, 6дБ, 790-2700 МГц, 4.3-10F, -160дБн, IP65 (Комбайнер 4х4, 8 портов)</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>Гибрид 4×4, 8 портов; 790–2700 МГц; 6 дБ; 4.3-10F; IP65. Изоляция и допустимая мощность не даны.</t>
         </is>
@@ -643,12 +649,12 @@
           <t>АФУ</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>PC250_Делитель мощности, 2:1, 700-2700 МГц, 4.3-10F, -160дБн, IP65</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>Делитель 2:1; 700–2700 МГц; 4.3-10F; IP65. Идеальное деление 3,01 дБ, excess loss не дано.</t>
         </is>
@@ -668,12 +674,12 @@
           <t>АФУ</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>PC252_Делитель мощности, 4:1, 700-2700 МГц, 4.3-10F, -160дБн, IP65</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>Делитель 4:1; 700–2700 МГц; 4.3-10F; IP65. Идеальное деление 6,02 дБ, excess loss не дано.</t>
         </is>
@@ -693,12 +699,12 @@
           <t>АФУ</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Фидер коаксиальный 1/2 гибкий, оболочка - огнестойкая безгалогеновая</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>1/2, 50 Ом по PDF LCF12-50J; 10,09 / 10,99 / 12,3867 дБ/100м при 1800/2100/2600 (последние две интерполированы). Пожарная модификация не подтверждена.</t>
         </is>
@@ -718,12 +724,12 @@
           <t>АФУ</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Фидер коаксиальный 7/8 гибкий, оболочка - огнестойкая безгалогеновая</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>7/8, 50 Ом по PDF LCF78-50JA-A0; 5,21 / 5,67 / 6,39 дБ/100м при 1800/2100/2600; допуск ±5%. Пожарная модификация не подтверждена.</t>
         </is>
@@ -748,7 +754,7 @@
           <t xml:space="preserve">Разъем 4.3-10 для 1/2 </t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>4.3-10 для фидера 1/2. Loss, PIM и конкретная модификация не предоставлены.</t>
         </is>
@@ -773,7 +779,7 @@
           <t>Разъем 4.3-10 для 7/8</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>4.3-10 для фидера 7/8. Loss, PIM и конкретная модификация не предоставлены.</t>
         </is>
@@ -798,7 +804,7 @@
           <t>Джамп-кабель 4.3-10m / 4.3-10m 3м</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>4.3-10 male / 4.3-10 male, 3 м. Собственное затухание и тип кабеля не предоставлены.</t>
         </is>
@@ -1023,7 +1029,7 @@
       <c r="B2" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="10" t="inlineStr">
         <is>
           <t>50 Ом; модели и допустимые мощности не предоставлены, в основную спецификацию не добавлены</t>
         </is>
@@ -1038,7 +1044,7 @@
       <c r="B3" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>Четвёртые входы гибридов B1/B7; отдельного резерва GSM О2/О3 нет</t>
         </is>
@@ -1055,7 +1061,7 @@
           <t>34 male + 34 female</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>Это требуемые исполнения в рамках общей позиции перечня; доступность не подтверждена</t>
         </is>
@@ -1072,7 +1078,7 @@
           <t>70 male + 30 female</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>Female на антенных концах для male/male джамперов; переходники не выдуманы</t>
         </is>
@@ -1089,7 +1095,7 @@
           <t>Интерфейс не задан</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>4.3-10F на In06 принят как условие стыковки, не характеристика из перечня</t>
         </is>
@@ -1106,7 +1112,7 @@
           <t>Условно общий RF-порт БС</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>При раздельных выходах нужно дополнительное решение; его модели нет в исходных данных</t>
         </is>
@@ -1123,7 +1129,7 @@
           <t>Отдельных входов нет</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>Три LTE-оператора предусмотрены, полное трёхоператорское использование GSM не подтверждено</t>
         </is>
@@ -1152,12 +1158,12 @@
           <t>PIM −160дБн</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Заявлено для пассивных компонентов в перечне</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>Условия измерения, допустимая суммарная мощность и изоляция не предоставлены</t>
         </is>
@@ -1169,12 +1175,12 @@
           <t>Пожарное исполнение</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>XLSX: огнестойкое, безгалогеновое; PDF: PE</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>Расчёт затухания по PDF не подтверждает требуемую модификацию</t>
         </is>
@@ -1243,7 +1249,7 @@
           <t>АФУ</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="10" t="inlineStr">
         <is>
           <t>In06_Потолочная, омни, MIMO, 800-2700 (G= 3dBi, H=360°)</t>
         </is>
@@ -1263,7 +1269,7 @@
           <t>АФУ</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>In08_Панельная настенная, MIMO (G=7dBi, H=90°, V=60°)</t>
         </is>
@@ -1283,7 +1289,7 @@
           <t>АФУ</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>PC211 Триплексер 1710-1880/1920-2170/2500-2690 МГц, одинарный, 4.3-10F, -160дБн, IP67</t>
         </is>
@@ -1303,7 +1309,7 @@
           <t>АФУ</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>PC221_Гибридный комбайнер, 6дБ, 790-2700 МГц, 4.3-10F, -160дБн, IP65 (Комбайнер 4х4, 8 портов)</t>
         </is>
@@ -1323,7 +1329,7 @@
           <t>АФУ</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>PC250_Делитель мощности, 2:1, 700-2700 МГц, 4.3-10F, -160дБн, IP65</t>
         </is>
@@ -1343,7 +1349,7 @@
           <t>АФУ</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>PC251_Делитель мощности, 3:1, 700-2700 МГц, 4.3-10F, -160дБн, IP65</t>
         </is>
@@ -1363,7 +1369,7 @@
           <t>АФУ</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>PC252_Делитель мощности, 4:1, 700-2700 МГц, 4.3-10F, -160дБн, IP65</t>
         </is>
@@ -1383,7 +1389,7 @@
           <t>АФУ</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>PC241_Направленный ответвитель, 7 dB,  700-2700 Мгц, 4.3-10F, -160дБн, IP65</t>
         </is>
@@ -1403,7 +1409,7 @@
           <t>АФУ</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>PC243_Направленный ответвитель, 10 dB,  700-2700 Мгц, 4.3-10F, -160дБн, IP65</t>
         </is>
@@ -1423,7 +1429,7 @@
           <t>АФУ</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>PC244_Направленный ответвитель, 13 dB,  700-2700 Мгц, 4.3-10F, -160дБн, IP65</t>
         </is>
@@ -1443,7 +1449,7 @@
           <t>АФУ</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>PC245_Направленный ответвитель, 15 dB,  700-2700 Мгц, 4.3-10F, -160дБн, IP65</t>
         </is>
@@ -1463,7 +1469,7 @@
           <t>АФУ</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="11" t="inlineStr">
         <is>
           <t>Фидер коаксиальный 1/2 гибкий, оболочка - огнестойкая безгалогеновая</t>
         </is>
@@ -1483,7 +1489,7 @@
           <t>АФУ</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>Фидер коаксиальный 7/8 гибкий, оболочка - огнестойкая безгалогеновая</t>
         </is>
@@ -1602,7 +1608,7 @@
           <t>Проект</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="10" t="inlineStr">
         <is>
           <t>Расчётный вариант финала с явно указанными ограничениями; не комплект для закупки без проверки паспортов и условий монтажа</t>
         </is>
@@ -1614,7 +1620,7 @@
           <t>32 антенн</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Проектные точки выбраны из CAD-привязок и сравнения покрытия. Координаты, распределение и исходные IDs — в project-input.json. Помещение 89 не локализовано.</t>
         </is>
@@ -1626,7 +1632,7 @@
           <t>Дерево на одну MIMO-ветвь</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>PC221: 4 выхода → 4 PC211 → 4 зоны. В каждой зоне PC252: два выхода напрямую на две антенны; третий через PC250 на две; четвёртый через PC252 на четыре. Доли мощности 1/4, 1/8, 1/16; 2+2+4=8 антенн.</t>
         </is>
@@ -1638,7 +1644,7 @@
           <t>PC221</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>6: 3 диапазона × 2 MIMO-ветви. По три входа для операторов; четвёртый B3 для GSM МТС. Все четыре выхода используются. Неизвестные мощности других операторов не подставлены.</t>
         </is>
@@ -1650,7 +1656,7 @@
           <t>PC250</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>9: один делит DCS-пул на два гибрида B3; восемь питают парные подгруппы, по одному на зону/ветвь.</t>
         </is>
@@ -1662,7 +1668,7 @@
           <t>PC211</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>8: 4 группы × 2 MIMO-ветви, по одному объединению B3/B1/B7 на каждый головной фидер</t>
         </is>
@@ -1674,7 +1680,7 @@
           <t>Фидеры</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>7/8 — все головные и подгрупповые участки и оконечные длиннее 15 м; 1/2 — короткие оконечные. Метраж схемы ×2 MIMO, затем +10% отдельного закупочного резерва. Правило 15 м — проектное решение, джамперы отдельно.</t>
         </is>
@@ -1686,7 +1692,7 @@
           <t>Разъёмы</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>По два на каждый ненулевой изготовляемый участок фидера. Для связи с male/male джампером оконечный разъём фидера должен быть female; у делителя — male. Пол разъёмов 1/2 и 7/8 в перечне не задан, доступность модификаций не подтверждена. Интерфейсы БС и In06 также не указаны.</t>
         </is>
@@ -1698,7 +1704,7 @@
           <t>113 джамперов</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>18 входов LTE + 1 вход GSM + 2 связи после PC250 + 24 связи PC221→PC211 + 64 антенных + 4 местных связей S→Q. При подключённом только МТС 12 входных связей зарезервированы. Порты БС и пригодность длины 3 м не подтверждены.</t>
         </is>
@@ -1710,7 +1716,7 @@
           <t>Местные связи</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>4 местных соединений: геометрическая длина 0 м означает соседние устройства; соединение выполнено джампером 3 м, по два на ID для MIMO. Добавлено 0,2 дБ на путь, собственное допущение. Монтажные фидеры и отдельные разъёмы для этих связей не считаются.</t>
         </is>
@@ -1722,7 +1728,7 @@
           <t>GSM-интерфейс</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Один общий RF-выход GSM с двумя TRX принят условно: объединение передатчиков внутри БС не подтверждено. При раздельных RF-выходах требуется дополнительное решение объединения, отсутствующее в исходных данных. Отдельные входы DCS двух других операторов не выделены.</t>
         </is>
@@ -1734,7 +1740,7 @@
           <t>Неиспользуемые порты</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>У B1/B7 гибридов остаются 4 незадействованных входа, а до подключения других операторов ещё 12. Нужны согласованные 50-омные нагрузки: их нет в разрешённом перечне; это открытое несоответствие, не выдуманная позиция спецификации.</t>
         </is>
@@ -1746,7 +1752,7 @@
           <t>Потери компонентов</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Кроме 6 дБ PC221 и идеального деления паспортные потери не заданы. Использованы сценарные оценки, см. RF-лист.</t>
         </is>
@@ -1758,7 +1764,7 @@
           <t>Пожарное исполнение</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>XLSX требует огнестойкую безгалогеновую оболочку; PDF описывают PE-варианты. Нужна допустимая модификация.</t>
         </is>
@@ -1770,7 +1776,7 @@
           <t>ВК</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>Проектная координата (9.2, 31.2); существующая ВК в DWG не найдена. Выделение части 104.2 под аппаратную — собственное решение, не исходное назначение комнаты.</t>
         </is>
@@ -1782,7 +1788,7 @@
           <t>Удалённое управление</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>В перечне нет подходящих управляемых модулей. Пассивная схема не подтверждает требование регулировки на удалённых модулях.</t>
         </is>
@@ -1874,7 +1880,7 @@
       <c r="E2" s="5" t="n">
         <v>28.4397</v>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="10" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -1900,7 +1906,7 @@
       <c r="E3" s="7" t="n">
         <v>28.1914</v>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F3" s="11" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -1926,7 +1932,7 @@
       <c r="E4" s="5" t="n">
         <v>15.6385</v>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="10" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -1952,7 +1958,7 @@
       <c r="E5" s="7" t="n">
         <v>61.9612</v>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="11" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -1978,7 +1984,7 @@
       <c r="E6" s="5" t="n">
         <v>5.6192</v>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="10" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2004,7 +2010,7 @@
       <c r="E7" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="11" t="inlineStr">
         <is>
           <t>Соседние устройства: два заводских джампера по 3 м; не нулевой фидер</t>
         </is>
@@ -2030,7 +2036,7 @@
       <c r="E8" s="5" t="n">
         <v>0.4444</v>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="10" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2056,7 +2062,7 @@
       <c r="E9" s="7" t="n">
         <v>36.4366</v>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="11" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2082,7 +2088,7 @@
       <c r="E10" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" s="10" t="inlineStr">
         <is>
           <t>Соседние устройства: два заводских джампера по 3 м; не нулевой фидер</t>
         </is>
@@ -2108,7 +2114,7 @@
       <c r="E11" s="7" t="n">
         <v>16.5322</v>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F11" s="11" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2134,7 +2140,7 @@
       <c r="E12" s="5" t="n">
         <v>27.4515</v>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F12" s="10" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2160,7 +2166,7 @@
       <c r="E13" s="7" t="n">
         <v>11.5469</v>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="F13" s="11" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2186,7 +2192,7 @@
       <c r="E14" s="5" t="n">
         <v>18.6482</v>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F14" s="10" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2212,7 +2218,7 @@
       <c r="E15" s="7" t="n">
         <v>25.2522</v>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="F15" s="11" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2238,7 +2244,7 @@
       <c r="E16" s="5" t="n">
         <v>38.8312</v>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F16" s="10" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2264,7 +2270,7 @@
       <c r="E17" s="7" t="n">
         <v>45.6789</v>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F17" s="11" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2290,7 +2296,7 @@
       <c r="E18" s="5" t="n">
         <v>101.9669</v>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="F18" s="10" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2316,7 +2322,7 @@
       <c r="E19" s="7" t="n">
         <v>8.978899999999999</v>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F19" s="11" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2342,7 +2348,7 @@
       <c r="E20" s="5" t="n">
         <v>3.3051</v>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F20" s="10" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2368,7 +2374,7 @@
       <c r="E21" s="7" t="n">
         <v>78.9036</v>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="F21" s="11" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2394,7 +2400,7 @@
       <c r="E22" s="5" t="n">
         <v>74.8171</v>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="F22" s="10" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2420,7 +2426,7 @@
       <c r="E23" s="7" t="n">
         <v>8.8942</v>
       </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="F23" s="11" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2446,7 +2452,7 @@
       <c r="E24" s="5" t="n">
         <v>73.27679999999999</v>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="F24" s="10" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2472,7 +2478,7 @@
       <c r="E25" s="7" t="n">
         <v>52.7212</v>
       </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="F25" s="11" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2498,7 +2504,7 @@
       <c r="E26" s="5" t="n">
         <v>17.9207</v>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="F26" s="10" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2524,7 +2530,7 @@
       <c r="E27" s="7" t="n">
         <v>57.066</v>
       </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="F27" s="11" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2550,7 +2556,7 @@
       <c r="E28" s="5" t="n">
         <v>1.2682</v>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="F28" s="10" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2576,7 +2582,7 @@
       <c r="E29" s="7" t="n">
         <v>10.6708</v>
       </c>
-      <c r="F29" s="6" t="inlineStr">
+      <c r="F29" s="11" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2602,7 +2608,7 @@
       <c r="E30" s="5" t="n">
         <v>13.8075</v>
       </c>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="F30" s="10" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2628,7 +2634,7 @@
       <c r="E31" s="7" t="n">
         <v>6.8864</v>
       </c>
-      <c r="F31" s="6" t="inlineStr">
+      <c r="F31" s="11" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2654,7 +2660,7 @@
       <c r="E32" s="5" t="n">
         <v>14.127</v>
       </c>
-      <c r="F32" s="4" t="inlineStr">
+      <c r="F32" s="10" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2680,7 +2686,7 @@
       <c r="E33" s="7" t="n">
         <v>43.8618</v>
       </c>
-      <c r="F33" s="6" t="inlineStr">
+      <c r="F33" s="11" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2706,7 +2712,7 @@
       <c r="E34" s="5" t="n">
         <v>5.3998</v>
       </c>
-      <c r="F34" s="4" t="inlineStr">
+      <c r="F34" s="10" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2732,7 +2738,7 @@
       <c r="E35" s="7" t="n">
         <v>12.3759</v>
       </c>
-      <c r="F35" s="6" t="inlineStr">
+      <c r="F35" s="11" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2758,7 +2764,7 @@
       <c r="E36" s="5" t="n">
         <v>33.9558</v>
       </c>
-      <c r="F36" s="4" t="inlineStr">
+      <c r="F36" s="10" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2784,7 +2790,7 @@
       <c r="E37" s="7" t="n">
         <v>7.77</v>
       </c>
-      <c r="F37" s="6" t="inlineStr">
+      <c r="F37" s="11" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2810,7 +2816,7 @@
       <c r="E38" s="5" t="n">
         <v>1.8352</v>
       </c>
-      <c r="F38" s="4" t="inlineStr">
+      <c r="F38" s="10" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2836,7 +2842,7 @@
       <c r="E39" s="7" t="n">
         <v>91.08629999999999</v>
       </c>
-      <c r="F39" s="6" t="inlineStr">
+      <c r="F39" s="11" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2862,7 +2868,7 @@
       <c r="E40" s="5" t="n">
         <v>5.0656</v>
       </c>
-      <c r="F40" s="4" t="inlineStr">
+      <c r="F40" s="10" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2888,7 +2894,7 @@
       <c r="E41" s="7" t="n">
         <v>118.3848</v>
       </c>
-      <c r="F41" s="6" t="inlineStr">
+      <c r="F41" s="11" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2914,7 +2920,7 @@
       <c r="E42" s="5" t="n">
         <v>64.38630000000001</v>
       </c>
-      <c r="F42" s="4" t="inlineStr">
+      <c r="F42" s="10" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2940,7 +2946,7 @@
       <c r="E43" s="7" t="n">
         <v>70.38939999999999</v>
       </c>
-      <c r="F43" s="6" t="inlineStr">
+      <c r="F43" s="11" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2966,7 +2972,7 @@
       <c r="E44" s="5" t="n">
         <v>0.1325</v>
       </c>
-      <c r="F44" s="4" t="inlineStr">
+      <c r="F44" s="10" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -2992,7 +2998,7 @@
       <c r="E45" s="7" t="n">
         <v>63.7964</v>
       </c>
-      <c r="F45" s="6" t="inlineStr">
+      <c r="F45" s="11" t="inlineStr">
         <is>
           <t>Проектная аппроксимация CAD-лотков; без запаса</t>
         </is>
@@ -11969,7 +11975,7 @@
       </c>
     </row>
     <row r="14" ht="51" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>P1_closed_gaps_geometry_uncertain_fail_RF3</t>
         </is>
@@ -12372,7 +12378,7 @@
       </c>
     </row>
     <row r="27" ht="51" customHeight="1">
-      <c r="A27" s="6" t="inlineStr">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>P1_closed_gaps_geometry_uncertain_fail_RF3</t>
         </is>
@@ -12775,7 +12781,7 @@
       </c>
     </row>
     <row r="40" ht="51" customHeight="1">
-      <c r="A40" s="4" t="inlineStr">
+      <c r="A40" s="10" t="inlineStr">
         <is>
           <t>P1_closed_gaps_geometry_uncertain_fail_RF3</t>
         </is>
@@ -18608,7 +18614,7 @@
       <c r="D2" s="5" t="n">
         <v>31.2</v>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="10" t="inlineStr">
         <is>
           <t>Головной узел; размеры и монтажная раскладка не заданы</t>
         </is>
@@ -18631,7 +18637,7 @@
       <c r="D3" s="7" t="n">
         <v>31.2</v>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>Головной узел; размеры и монтажная раскладка не заданы</t>
         </is>
@@ -18654,7 +18660,7 @@
       <c r="D4" s="5" t="n">
         <v>31.2</v>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>Головной узел; размеры и монтажная раскладка не заданы</t>
         </is>
@@ -18723,7 +18729,7 @@
       <c r="D7" s="7" t="n">
         <v>46.02057642602261</v>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="11" t="inlineStr">
         <is>
           <t>Подгруппа на трассе; M1/M2 показаны одной геометрической точкой</t>
         </is>
@@ -18746,7 +18752,7 @@
       <c r="D8" s="5" t="n">
         <v>43.21100027232224</v>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>Подгруппа на трассе; M1/M2 показаны одной геометрической точкой</t>
         </is>
@@ -18815,7 +18821,7 @@
       <c r="D11" s="7" t="n">
         <v>30.542096</v>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="11" t="inlineStr">
         <is>
           <t>Подгруппа на трассе; M1/M2 показаны одной геометрической точкой</t>
         </is>
@@ -18838,7 +18844,7 @@
       <c r="D12" s="5" t="n">
         <v>39.986112</v>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>Подгруппа на трассе; M1/M2 показаны одной геометрической точкой</t>
         </is>
@@ -18907,7 +18913,7 @@
       <c r="D15" s="7" t="n">
         <v>26.486112</v>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E15" s="11" t="inlineStr">
         <is>
           <t>Подгруппа на трассе; M1/M2 показаны одной геометрической точкой</t>
         </is>
@@ -18930,7 +18936,7 @@
       <c r="D16" s="5" t="n">
         <v>28.115735</v>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>Подгруппа на трассе; M1/M2 показаны одной геометрической точкой</t>
         </is>
@@ -18999,7 +19005,7 @@
       <c r="D19" s="7" t="n">
         <v>4.584693</v>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E19" s="11" t="inlineStr">
         <is>
           <t>Подгруппа на трассе; M1/M2 показаны одной геометрической точкой</t>
         </is>
@@ -19022,7 +19028,7 @@
       <c r="D20" s="5" t="n">
         <v>10.8684375</v>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E20" s="10" t="inlineStr">
         <is>
           <t>Подгруппа на трассе; M1/M2 показаны одной геометрической точкой</t>
         </is>
@@ -19045,7 +19051,7 @@
       <c r="D21" s="7" t="n">
         <v>31.2</v>
       </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>Головной узел; размеры и монтажная раскладка не заданы</t>
         </is>
@@ -19068,7 +19074,7 @@
       <c r="D22" s="5" t="n">
         <v>31.2</v>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E22" s="10" t="inlineStr">
         <is>
           <t>Головной узел; размеры и монтажная раскладка не заданы</t>
         </is>
@@ -19091,7 +19097,7 @@
       <c r="D23" s="7" t="n">
         <v>31.2</v>
       </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="E23" s="11" t="inlineStr">
         <is>
           <t>Головной узел; размеры и монтажная раскладка не заданы</t>
         </is>
@@ -19160,7 +19166,7 @@
       <c r="D26" s="5" t="n">
         <v>46.02057642602261</v>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" s="10" t="inlineStr">
         <is>
           <t>Подгруппа на трассе; M1/M2 показаны одной геометрической точкой</t>
         </is>
@@ -19183,7 +19189,7 @@
       <c r="D27" s="7" t="n">
         <v>43.21100027232224</v>
       </c>
-      <c r="E27" s="6" t="inlineStr">
+      <c r="E27" s="11" t="inlineStr">
         <is>
           <t>Подгруппа на трассе; M1/M2 показаны одной геометрической точкой</t>
         </is>
@@ -19252,7 +19258,7 @@
       <c r="D30" s="5" t="n">
         <v>30.542096</v>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="E30" s="10" t="inlineStr">
         <is>
           <t>Подгруппа на трассе; M1/M2 показаны одной геометрической точкой</t>
         </is>
@@ -19275,7 +19281,7 @@
       <c r="D31" s="7" t="n">
         <v>39.986112</v>
       </c>
-      <c r="E31" s="6" t="inlineStr">
+      <c r="E31" s="11" t="inlineStr">
         <is>
           <t>Подгруппа на трассе; M1/M2 показаны одной геометрической точкой</t>
         </is>
@@ -19344,7 +19350,7 @@
       <c r="D34" s="5" t="n">
         <v>26.486112</v>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="E34" s="10" t="inlineStr">
         <is>
           <t>Подгруппа на трассе; M1/M2 показаны одной геометрической точкой</t>
         </is>
@@ -19367,7 +19373,7 @@
       <c r="D35" s="7" t="n">
         <v>28.115735</v>
       </c>
-      <c r="E35" s="6" t="inlineStr">
+      <c r="E35" s="11" t="inlineStr">
         <is>
           <t>Подгруппа на трассе; M1/M2 показаны одной геометрической точкой</t>
         </is>
@@ -19436,7 +19442,7 @@
       <c r="D38" s="5" t="n">
         <v>4.584693</v>
       </c>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="E38" s="10" t="inlineStr">
         <is>
           <t>Подгруппа на трассе; M1/M2 показаны одной геометрической точкой</t>
         </is>
@@ -19459,7 +19465,7 @@
       <c r="D39" s="7" t="n">
         <v>10.8684375</v>
       </c>
-      <c r="E39" s="6" t="inlineStr">
+      <c r="E39" s="11" t="inlineStr">
         <is>
           <t>Подгруппа на трассе; M1/M2 показаны одной геометрической точкой</t>
         </is>
@@ -19505,7 +19511,7 @@
       <c r="D41" s="7" t="n">
         <v>49.02438226281524</v>
       </c>
-      <c r="E41" s="6" t="inlineStr">
+      <c r="E41" s="11" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -19528,7 +19534,7 @@
       <c r="D42" s="5" t="n">
         <v>55</v>
       </c>
-      <c r="E42" s="4" t="inlineStr">
+      <c r="E42" s="10" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -19551,7 +19557,7 @@
       <c r="D43" s="7" t="n">
         <v>63.42404058032748</v>
       </c>
-      <c r="E43" s="6" t="inlineStr">
+      <c r="E43" s="11" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -19574,7 +19580,7 @@
       <c r="D44" s="5" t="n">
         <v>59.99460955452709</v>
       </c>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="E44" s="10" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -19597,7 +19603,7 @@
       <c r="D45" s="7" t="n">
         <v>49.02438226281524</v>
       </c>
-      <c r="E45" s="6" t="inlineStr">
+      <c r="E45" s="11" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -19620,7 +19626,7 @@
       <c r="D46" s="5" t="n">
         <v>46.02057642602261</v>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="E46" s="10" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -19643,7 +19649,7 @@
       <c r="D47" s="7" t="n">
         <v>43.21100027232224</v>
       </c>
-      <c r="E47" s="6" t="inlineStr">
+      <c r="E47" s="11" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -19666,7 +19672,7 @@
       <c r="D48" s="5" t="n">
         <v>40.21100027232223</v>
       </c>
-      <c r="E48" s="4" t="inlineStr">
+      <c r="E48" s="10" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -19689,7 +19695,7 @@
       <c r="D49" s="7" t="n">
         <v>50.48999999999999</v>
       </c>
-      <c r="E49" s="6" t="inlineStr">
+      <c r="E49" s="11" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -19712,7 +19718,7 @@
       <c r="D50" s="5" t="n">
         <v>26.095</v>
       </c>
-      <c r="E50" s="4" t="inlineStr">
+      <c r="E50" s="10" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -19735,7 +19741,7 @@
       <c r="D51" s="7" t="n">
         <v>60.20952398557016</v>
       </c>
-      <c r="E51" s="6" t="inlineStr">
+      <c r="E51" s="11" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -19758,7 +19764,7 @@
       <c r="D52" s="5" t="n">
         <v>33.62879322850282</v>
       </c>
-      <c r="E52" s="4" t="inlineStr">
+      <c r="E52" s="10" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -19781,7 +19787,7 @@
       <c r="D53" s="7" t="n">
         <v>47.28251056928649</v>
       </c>
-      <c r="E53" s="6" t="inlineStr">
+      <c r="E53" s="11" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -19804,7 +19810,7 @@
       <c r="D54" s="5" t="n">
         <v>46.83554124130971</v>
       </c>
-      <c r="E54" s="4" t="inlineStr">
+      <c r="E54" s="10" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -19827,7 +19833,7 @@
       <c r="D55" s="7" t="n">
         <v>40.62021820570461</v>
       </c>
-      <c r="E55" s="6" t="inlineStr">
+      <c r="E55" s="11" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -19850,7 +19856,7 @@
       <c r="D56" s="5" t="n">
         <v>35.32850186609248</v>
       </c>
-      <c r="E56" s="4" t="inlineStr">
+      <c r="E56" s="10" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -19873,7 +19879,7 @@
       <c r="D57" s="7" t="n">
         <v>20.56811553916096</v>
       </c>
-      <c r="E57" s="6" t="inlineStr">
+      <c r="E57" s="11" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -19896,7 +19902,7 @@
       <c r="D58" s="5" t="n">
         <v>30.86086281460469</v>
       </c>
-      <c r="E58" s="4" t="inlineStr">
+      <c r="E58" s="10" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -19919,7 +19925,7 @@
       <c r="D59" s="7" t="n">
         <v>23.56811553916096</v>
       </c>
-      <c r="E59" s="6" t="inlineStr">
+      <c r="E59" s="11" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -19942,7 +19948,7 @@
       <c r="D60" s="5" t="n">
         <v>21.26786214284159</v>
       </c>
-      <c r="E60" s="4" t="inlineStr">
+      <c r="E60" s="10" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -19965,7 +19971,7 @@
       <c r="D61" s="7" t="n">
         <v>30.792355587748</v>
       </c>
-      <c r="E61" s="6" t="inlineStr">
+      <c r="E61" s="11" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -19988,7 +19994,7 @@
       <c r="D62" s="5" t="n">
         <v>30.71789008037059</v>
       </c>
-      <c r="E62" s="4" t="inlineStr">
+      <c r="E62" s="10" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -20011,7 +20017,7 @@
       <c r="D63" s="7" t="n">
         <v>24.58</v>
       </c>
-      <c r="E63" s="6" t="inlineStr">
+      <c r="E63" s="11" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -20034,7 +20040,7 @@
       <c r="D64" s="5" t="n">
         <v>27.93276712019818</v>
       </c>
-      <c r="E64" s="4" t="inlineStr">
+      <c r="E64" s="10" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -20057,7 +20063,7 @@
       <c r="D65" s="7" t="n">
         <v>3.667097893003584</v>
       </c>
-      <c r="E65" s="6" t="inlineStr">
+      <c r="E65" s="11" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -20080,7 +20086,7 @@
       <c r="D66" s="5" t="n">
         <v>12.4507421875</v>
       </c>
-      <c r="E66" s="4" t="inlineStr">
+      <c r="E66" s="10" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -20103,7 +20109,7 @@
       <c r="D67" s="7" t="n">
         <v>17.345</v>
       </c>
-      <c r="E67" s="6" t="inlineStr">
+      <c r="E67" s="11" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -20126,7 +20132,7 @@
       <c r="D68" s="5" t="n">
         <v>21.87877117801221</v>
       </c>
-      <c r="E68" s="4" t="inlineStr">
+      <c r="E68" s="10" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -20149,7 +20155,7 @@
       <c r="D69" s="7" t="n">
         <v>4.16375</v>
       </c>
-      <c r="E69" s="6" t="inlineStr">
+      <c r="E69" s="11" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -20172,7 +20178,7 @@
       <c r="D70" s="5" t="n">
         <v>2.132269541326413</v>
       </c>
-      <c r="E70" s="4" t="inlineStr">
+      <c r="E70" s="10" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -20195,7 +20201,7 @@
       <c r="D71" s="7" t="n">
         <v>10.8684375</v>
       </c>
-      <c r="E71" s="6" t="inlineStr">
+      <c r="E71" s="11" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>
@@ -20218,7 +20224,7 @@
       <c r="D72" s="5" t="n">
         <v>5.653403907351852</v>
       </c>
-      <c r="E72" s="4" t="inlineStr">
+      <c r="E72" s="10" t="inlineStr">
         <is>
           <t>Исследовательская позиция n=3; монтажная доступность не подтверждена</t>
         </is>

</xml_diff>